<commit_message>
Note Ultratex key-person follow-up: still not found in public sources
Documented second-pass checks (DED licence republish, LinkedIn, email
databases, IATF directories, Arabic name, unrelated UK/China namesakes).
No invented contacts; files updated with research notes only.
</commit_message>
<xml_diff>
--- a/bots/服装外贸/丝路-背调开发信/deliverables/fabric_buyers_batch1_verified_2026-10-29.xlsx
+++ b/bots/服装外贸/丝路-背调开发信/deliverables/fabric_buyers_batch1_verified_2026-10-29.xlsx
@@ -1221,7 +1221,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://www.ultratextrading.com/ | https://overit.ae/company/ideally-textiles-trading-l-l-c</t>
+          <t>https://www.ultratextrading.com/ | https://overit.ae/company/ideally-textiles-trading-l-l-c | https://overit.ae/company/ideally-textiles-trading-l-l-c | IATF Directory May/Nov 2024–2025（无匹配） | LinkedIn domain lookup miss | Tomba/Anymailfinder domain email list empty</t>
         </is>
       </c>
       <c r="K10" s="4" t="n">
@@ -1234,17 +1234,17 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>公司已核实；关键人未找到；邮箱未验证</t>
+          <t>公司已核实；关键人二次深挖后仍未找到；邮箱未验证</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>用sales@发中国现货梭织/针织目录；同步在迪拜展会或WhatsApp补关键人。</t>
+          <t>付费调取迪拜DET执照完整摘要（股东/经理），或WhatsApp +971 50 525 0301先确认采购对接人；暂用sales@开发。</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>关键人姓名经官网、LinkedIn、UAE公开目录检索后仍未找到。</t>
+          <t>关键人姓名经官网、LinkedIn、UAE公开目录检索后仍未找到。 【2026-10-30二次深挖关键人】公开渠道仍未找到业主/董事/采购负责人姓名。已查：官网全文（无About/Team页，仅info@/sales@与电话）；迪拜DED执照881760经Overit转载（不公布股东/经理）；LinkedIn公司页未找到（domain-to-linkedin miss）；Tomba/Anymailfinder域名邮箱列表为空；IATF Dubai展商名录May/Nov 2024–2025全文检索无Ultratex；阿语名「التراتيكس」检索无经理/业主；英国Ultratex Trading Ltd（03347188，2013解散，董事Muhammed Uzair Malik）与迪拜主体无公开关联证据，未并入；绍兴Shaoxing Ultratex（Olga Yakuntseva/Debbie Chen）服务俄罗斯Ultratex缝纫辅料，与迪拜面料进口商无公开股权/雇佣关联证据，未并入。建议下一步：付费调取迪拜DET完整执照摘要（含managers/shareholders），或WhatsApp +971 50 525 0301询采购人姓名。</t>
         </is>
       </c>
     </row>

</xml_diff>